<commit_message>
Rewrite manuscript in Medicine-style structure; move extended content to supplement (S1-S16, Figures S1-S9); remove earlier manuscript versions
</commit_message>
<xml_diff>
--- a/results/Supplementary_Tables.xlsx
+++ b/results/Supplementary_Tables.xlsx
@@ -33,6 +33,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S10 Influence diagnostics" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S11 Radial MR" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12 Cross-dataset concordance" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13 Dataset characteristics" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14 Diagnostics summary" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15 Sensitivity analyses" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16 Positive control summary" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30668,6 +30672,642 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Design / source</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Variants used</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>R2 (%)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Mean F (min)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MDE, OR*</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exposure: RC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UK Biobank NMR GWAS (Richardson 2022); N = 115,082</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>150 (29.8)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ghodsian 2021</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EHR meta-analysis of 4 cohorts; GCST90091033</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>8,434</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>770,180</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>150 (29.8)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Fairfield 2022</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UK Biobank; GCST90054782</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4,761</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>373,227</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>147 (29.8)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FinnGen R5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FinnGen; finn-b-NAFLD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>894</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>217,898</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>150 (29.8)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Positive control: CAD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CARDIoGRAMplusC4D 1000G (Nikpay 2015); GCST003116</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>60,801</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>123,504</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>150 (29.8)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SNPs</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>QIVW (P)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>I2 (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>I2GX (%)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Egger intercept (P)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>MR-PRESSO outliers</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Radial outliers</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Cook &gt; 4/n</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ghodsian</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>204.8 (1.4 × 10−21)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>77.1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>99.3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.0112 (.261)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>rs112875651, rs58542926, rs4665972, rs2326077</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fairfield</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>251.4 (1.2 × 10−28)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>80.1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>99.3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.0211 (.118)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>rs112875651, rs58542926, rs4665972</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FinnGen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>106.2 (1.8 × 10−6)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>55.7</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>99.3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>−0.0013 (.952)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>rs112875651, rs58542926</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ghodsian: OR (95% CI), P</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Fairfield: OR (95% CI), P</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>FinnGen: OR (95% CI), P</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>All variants</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1.045 (0.864–1.265), .650 [48]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.999 (0.776–1.286), .994 [51]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.848 (0.561–1.281), .433 [48]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MR-PRESSO outliers removed</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.023 (0.914–1.145), .695 [44]</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.009 (0.871–1.169), .908 [48]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.839 (0.624–1.127), .250 [46]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Steiger-filtered</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.081 (0.943–1.238), .263 [45]</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.996 (0.865–1.146), .951 [47]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.949 (0.706–1.275), .727 [35]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>APOE region excluded</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.073 (0.853–1.349), .548 [45]</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.014 (0.748–1.374), .930 [47]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.859 (0.539–1.369), .523 [45]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F ≥ 30 only</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.046 (0.862–1.269), .648 [47]</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.993 (0.770–1.280), .958 [50]</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.861 (0.570–1.301), .478 [47]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Earlier 48-variant set</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.984 (0.869–1.114), .798 [41]</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.990 (0.851–1.152), .898 [48]</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.752 (0.562–1.006), .055 [43]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -34267,6 +34907,209 @@
       </c>
       <c r="T52" t="n">
         <v>0.0001630063367049</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SNPs</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>IVW</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1.579</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1.378–1.809</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5.2 × 10−11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MR-Egger</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.871</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1.461–2.395</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>9.4 × 10−6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Weighted median</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.475</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1.321–1.648</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5.6 × 10−12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Simple mode</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.408</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1.088–1.821</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>.012</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Weighted mode</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.393</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.216–1.597</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.7 × 10−5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IVW after MR-PRESSO outlier removal (R)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1.492</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1.348–1.651</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.4 × 10−9</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>